<commit_message>
Added Web Page and Email feature works on my machine
</commit_message>
<xml_diff>
--- a/applications.xlsx
+++ b/applications.xlsx
@@ -413,12 +413,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
@@ -465,48 +465,52 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Veracyte</t>
+          <t>Autoliv</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Intern, AI (PMO)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>Gen AI intern</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Auburn Hills, Michigan</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>applied</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
+          <t>interview_invite</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Thank you for applying to Veracyte</t>
+          <t>RE: Thank you for Interview</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Application received confirmation for AI PMO internship position</t>
+          <t>Interview invitation with specific interviewer (Venkatesh Vallapureddy, Development Senior Engineer, GDA Buckles)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Menasha Corporation</t>
+          <t>Aquatic Capital Management</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Application Engineer Intern</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>Software Engineer, Intern (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>applied</t>
@@ -514,76 +518,64 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Application Received for Application Engineer Intern (Fall/Winter 2026)</t>
+          <t>Application Update |  Software Engineer, Intern (Summer 2027)  - Aquatic Capital Management</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Application received confirmation for Fall/Winter 2026 internship position</t>
+          <t>Application received confirmation from Greenhouse ATS</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Accel Learning</t>
+          <t>Maroon</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AI Engineer (Internship) - Intelligent Question Bank Platform</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Secaucus, NJ</t>
+          <t>Columbia, Maryland</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>applied</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
+          <t>interview_invite</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>We have received your application</t>
+          <t>Re: Invitation to Interview with Maroon</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Application received confirmation from Accel Learning via SmartRecruiters</t>
+          <t>Interview invitation with alignment check before scheduling; 2-3 hours/week, 5 weeks internship</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NextGen Federal Systems</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Data Science &amp; Machine Learning Intern</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
+          <t>D. E. Shaw Group</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>applied</t>
+          <t>follow_up</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -593,60 +585,68 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Thank you for your application to NextGen Federal Systems</t>
+          <t>From the D. E. Shaw group</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Application receipt confirmation from Lever hiring platform</t>
+          <t>Application review response indicating no current position match, appears to be a rejection or holding pattern</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>D. E. Shaw Group</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
+          <t>ZF</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Digitization Intern</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>New York, New York</t>
+          <t>Marysville</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>applied</t>
+          <t>follow_up</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Your application to the D. E. Shaw group</t>
+          <t>Re: ZF Digitization Intern - Marysville</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Application receipt confirmation from recruiting team</t>
+          <t>Personal message from recruiter at ZF acknowledging application to internship position</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Danaher</t>
+          <t>Veracyte</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Digital Analyst Internships</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>Intern, AI (PMO)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>applied</t>
@@ -659,29 +659,29 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Congrats on your application for the Digital Analyst Internships at Danaher!</t>
+          <t>Thank you for applying to Veracyte</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Application confirmation email from WayUp for Danaher Digital Analyst Internships role</t>
+          <t>Application confirmation email for Intern, AI (PMO) position</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CTGT</t>
+          <t>Menasha Corporation</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>Application Engineer Intern</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Troy, MI</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -696,29 +696,29 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Your application for CTGT - Software Engineering Intern (Summer 2027)</t>
+          <t>Application Received for Application Engineer Intern (Fall/Winter 2026)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Application confirmation email from Y Combinator Work at a Startup platform for Summer 2027 internship</t>
+          <t>Application received confirmation from Menasha Corporation for Fall/Winter 2026 intern position</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Citadel</t>
+          <t>Accel Learning</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Software Engineer - Intern</t>
+          <t>AI Engineer (Internship) - Intelligent Question Bank Platform</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Secaucus, NJ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -733,27 +733,31 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Your application for Citadel's Software Engineer - Intern (US) role has been received.</t>
+          <t>We have received your application</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Application receipt confirmation from Citadel hiring team</t>
+          <t>Application received confirmation from Accel Learning via SmartRecruiters</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Aquatic Capital Management</t>
+          <t>NextGen Federal Systems</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Claude Corps Fellowship</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>Data Science &amp; Machine Learning Intern</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>applied</t>
@@ -766,27 +770,31 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Thank you for applying to Aquatic Capital Management</t>
+          <t>Thank you for your application to NextGen Federal Systems</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Application received confirmation for Claude Corps Fellowship</t>
+          <t>Application received confirmation from Lever ATS system</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Anduril</t>
+          <t>Danaher</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2027 Software Engineer Intern</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>Digital Analyst Internships</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Edwardsville, Illinois</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>applied</t>
@@ -799,89 +807,105 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Your Application to Anduril</t>
+          <t>Congrats on your application for the Digital Analyst Internships at Danaher!</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Application received confirmation for Software Engineer Intern role</t>
+          <t>Application confirmation from WayUp Team confirming receipt and review status</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Freudenberg Sealing Technologies</t>
+          <t>Y Combinator (CTGT)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Engineering Intern</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>Software Engineering Intern</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>rejected</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Freudenberg-NOK Engineering Intern</t>
+          <t>Your application for CTGT - Software Engineering Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Rejection email for submitted engineering intern application</t>
+          <t>Application confirmation for Summer 2027 internship position</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Heard Sop</t>
+          <t>Citadel</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Startup Software Developer Intern</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>Software Engineer - Intern (US)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>interview_invite</t>
+          <t>applied</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Re: Next steps on your application</t>
+          <t>Your application for Citadel's Software Engineer - Intern (US) role has been received.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Direct recruiter/hiring manager invitation to schedule a call after reviewing application</t>
+          <t>Application received confirmation from Citadel hiring team</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cotiviti</t>
+          <t>Anduril</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Intern - AI Engineer</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>2027 Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Multiple: Atlanta, GA; Boston, MA; Costa Mesa, CA; Irvine, CA; Reston, VA; Seattle, WA</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
           <t>applied</t>
@@ -889,178 +913,198 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Thank you for applying at Cotiviti</t>
+          <t>Your Application to Anduril</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Application received confirmation from Cotiviti's automated system</t>
+          <t>Application received confirmation for Software Engineer Intern role</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Valeo</t>
+          <t>Freudenberg Sealing Technologies</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Systems Engineering Co-Op</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Troy, Michigan</t>
-        </is>
-      </c>
+          <t>Engineering Intern</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>applied</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>News about your application at Valeo for the Job Requisition - REQ2026070436 Systems Engineering Co-Op (Open)</t>
+          <t>Freudenberg-NOK Engineering Intern</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Application confirmation email from Valeo for Systems Engineering Co-Op position</t>
+          <t>Rejection notice for Engineering Intern position; email snippet cuts off but opening indicates negative decision</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>Heard Sop</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Intern, AI in Design &amp; Manufacturing</t>
+          <t>Startup Software Developer Intern</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>follow_up</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>interview_invite</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Update from Autodesk on 26WD94900 Intern, AI in Design &amp; Manufacturing (Open) &amp;#xa; Mise à jour d'Autodesk concernant la 26WD94900 Intern, AI in Design &amp; Manufacturing (Open)</t>
+          <t>Re: Next steps on your application</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Automated follow-up notification from Workday HR system about existing application</t>
+          <t>Direct interview invitation from hiring manager Dimitrios Provistalis following application review</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Frontline Education</t>
+          <t>Cotiviti</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>AI Operations Intern</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>Intern - AI Engineer</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>follow_up</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Re: Application for AI Operations Intern - Frontline Education</t>
+          <t>Thank you for applying at Cotiviti</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Update that they are interviewing for the position; appears to be a status notification rather than a direct interview invitation</t>
+          <t>Automatic application confirmation from Cotiviti's ATS system</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>Valeo</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Intern - Systems</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>Systems Engineering Co-Op</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Troy, MI</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>rejected</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Thank you for your Application!</t>
+          <t>News about your application at Valeo for the Job Requisition - REQ2026070436 Systems Engineering Co-Op (Open)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Rejection notice for submitted application</t>
+          <t>Application received confirmation from Valeo for Systems Engineering Co-Op position</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Autoliv</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
+          <t>Autodesk</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Intern, AI in Design &amp; Manufacturing</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>interview_invite</t>
+          <t>follow_up</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RE: Follow up on Phone Call with VP</t>
+          <t>Update from Autodesk on 26WD94900 Intern, AI in Design &amp; Manufacturing (Open) &amp;#xa; Mise à jour d'Autodesk concernant la 26WD94900 Intern, AI in Design &amp; Manufacturing (Open)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>In-person interview scheduled for Monday, July 13th with VP; follow-up to previous phone call</t>
+          <t>Automatic system notification following up on application status from Workday HR system</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Athena</t>
+          <t>Frontline Education</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>AI Engineering Intern</t>
+          <t>AI Operations Intern</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1069,15 +1113,1578 @@
           <t>follow_up</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
+          <t>Re: Application for AI Operations Intern - Frontline Education</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Update email indicating they are interviewing candidates; appears to be a follow-up rather than initial confirmation or interview invite</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Claude Corps Fellowship</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Your Claude Corps Fellowship application</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Application received confirmation for Claude Corps Fellowship</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Intern - Systems</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Thank you for your Application!</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Rejection email for Systems Intern position at MIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>AI Engineering Intern</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>follow_up</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>Athena: Application Status</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Follow-up email requesting completion of application questionnaire after initial application submission</t>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Application received but missing required attachments; needs resubmission</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Gen AI intern</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>follow_up</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Gen AI intern check up</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Candidate following up about a scheduled interview that had technical issues (no one joined the meeting)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Ededge Learning</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Data Analyst</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Data Analyst Training and Internship Program</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>LinkedIn application confirmation for Ededge Learning position</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BorgWarner</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern (Year-Round)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Auburn Hills, MI</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Thank you for Applying to BorgWarner</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Application receipt confirmation from BorgWarner HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Steel Services LTD</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>AI Intern</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>New York City, NY or Miami, FL</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Employment Update - Steel Services LTD</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Application received confirmation for AI Intern position</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Conquest Advisors</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Abbas, your application was sent to Conquest Advisors</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>LinkedIn confirmation that application was sent to Conquest Advisors</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Clinical Ink</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>AI &amp; Innovation Intern</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Thanks for Applying to Clinical Ink!</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Application receipt confirmation from Clinical Ink HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Statecraft Examiners, LLC</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Abbas, your application was sent to Statecraft Examiners, LLC</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>LinkedIn application confirmation for Statecraft Examiners, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Tessera Labs</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern, Frontend</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>San Jose, CA or Remote</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Thanks for applying to Tessera Labs!</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Application received confirmation from Tessera Labs hiring team</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Software Development Engineer Internship - Fall 2026 (US)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Thank you for Applying to Amazon!</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Application confirmation/receipt notification from Amazon careers portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Magna International</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Intern - Systems</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Southfield, Michigan</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>interview_invite</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Thanks for applying to the Intern - Systems - R00235414 at Magna International!</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Interview invitation from recruiter with Microsoft Teams meeting link</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Plexis Healthcare Systems</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Internship - AI Special Ops</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Application Received</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Application received confirmation with link to view/edit application</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Cohere</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (Fall/Winter, 2026)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Thanks for applying to Cohere!</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Application confirmation email from Cohere Talent Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Claude Corps</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>We received your Claude Corps application</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Application received confirmation from Greenhouse ATS system</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Actalent</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>We received your application</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Application confirmation from Actalent; awaiting recruiter review</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Aviator</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>GTM Engineering Intern</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Your application for Aviator - GTM Engineering Intern</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Application confirmation email from Y Combinator's job board for a specific role</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Kinaxis Inc.</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Co-op/Intern Information Security</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Your journey with Kinaxis starts here!</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Application received confirmation from Kinaxis talent system</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Virtual IP</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Abbas, your application was sent to Virtual IP</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>LinkedIn application confirmation for Virtual IP position</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Conduent</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Summer Intern – CXM Transformation, AI &amp; GTM Support</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Thank You for Applying at Conduent</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Application received confirmation for summer internship position</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>RevNet LLC</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Data Entry Intern</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Thank you for applying to RevNet LLC</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Application received confirmation from RevNet LLC hiring team</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>CPI Card Group</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Intern-AI Automation &amp; Process Analyst</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Thank you for your application</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Email verification request from applicant tracking system (iCIMS) - administrative step in application process</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>TechOnPurpose</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>AI Automation Architect (Intern)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Thank you for applying at TechOnPurpose</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Application received confirmation from TechOnPurpose via BambooHR</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Point C</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Thank you for applying to Point C!</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Application received confirmation from Greenhouse ATS system</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>AspiringIT</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Abbas, your application was sent to AspiringIT</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>LinkedIn notification confirming application was sent to AspiringIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ConnectPrep</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Data Analyst Internship</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Thanks for applying to ConnectPrep</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Application confirmation receipt from Workable system for Data Analyst Internship position</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Traackr</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern (Part-Time, Internal Tooling)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>New York City, NY</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Thanks for applying to Software Engineering Intern (Part-Time, Internal Tooling), here is a link to manage your application data</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Application received confirmation from Traackr via Lever hiring platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Bugcrowd</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Thank you for applying to Bugcrowd</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Application received confirmation from Greenhouse ATS</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Selkirk Sport</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Coeur d'Alene, ID</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Thank you for applying to Selkirk Sport</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Application received confirmation from Selkirk Sport ATS system</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>VetsEZ</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Full Stack Developer Intern</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Re: VetsEZ opportunity</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Rejection notice for Full Stack Developer Intern position; company offering to retain resume for future opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Clipboard</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Engineering Intern</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Your application for Clipboard - Engineering Intern</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Application confirmation from Y Combinator Work at a Startup platform for Clipboard Engineering Intern position</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Outmarket AI</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>AI Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Thanks for applying to Outmarket AI!</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Application received confirmation from hiring team</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Allus AI</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Software Engineer Internship</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Your application for Allus AI - Software Engineer Internship</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Application confirmation from Y Combinator Work at a Startup platform for Allus AI internship position</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>LG AI Research</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>[LG AI Research] Application Submitted!</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Application received confirmation from LG AI Research careers portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Innovaccer</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Abbas, your application was sent to Innovaccer</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>LinkedIn application confirmation notification</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Johnson Electric</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Thank you for your interest in Johnson Electric</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Application received confirmation from Johnson Electric via Workday</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ISUZU NORTH AMERICA CORPORATION</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>AI &amp; Autonomous Driving Intern</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>follow_up</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>ISUZU NORTH AMERICA CORPORATION Password setup</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Password setup email for applicant portal access after expressing interest in position</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>IT Co-Op</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Thank you for applying</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Application confirmation from SuccessFactors ATS system</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>American Heart Association</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Intern, Data Science</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>follow_up</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Thank You for Applying for the Intern, Data Science-Remote position at American Heart Association</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Follow-up reminder to complete application process on employer's site via WayUp platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>iHerb</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Thank You for Applying (iHerb Careers)</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Application received confirmation from iHerb Careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>CrowdStrike</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Intelligence</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Update on Your Recent CrowdStrike Job Application</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Rejection notice for application to CrowdStrike Intelligence position</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Allied Benefit Systems</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Software Engineering Apprentice</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>follow_up</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Your Software Engineering Apprentice Application</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Password setup email for new hire or onboarding system access, appears to be post-offer/acceptance stage</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Pulsewave</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Abbas, your application was sent to Pulsewave</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>LinkedIn application confirmation for Pulsewave</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Beyondsoft Consulting</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Thank you for your application</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Application received confirmation from ATS system</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Signal Advisors</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Internships 2026</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Thank you for applying- Signal Advisors</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Application received confirmation for internship role</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Affirm</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Software Engineering Apprentice, Full-Stack</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Thank you for your interest in Software Engineering Apprentice, Full-Stack at Affirm!</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Position filled; rejection notice for submitted application</t>
         </is>
       </c>
     </row>

</xml_diff>